<commit_message>
QA: Enlace de hipervinculos de GitHub a la matriz de control de versiones
</commit_message>
<xml_diff>
--- a/Matriz_Registro_Control_de_Versiones.xlsx
+++ b/Matriz_Registro_Control_de_Versiones.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,6 +69,13 @@
       <name val="Consolas"/>
       <color rgb="00212529"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="000d6efd"/>
+      <sz val="9"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="7">
@@ -135,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -161,6 +168,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -177,6 +187,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -698,7 +711,7 @@
           <t>main</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>0629d31</t>
         </is>
@@ -714,55 +727,55 @@
 0.23 ms Latencia de inferencia</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>APROBADO</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>BOLT-002-FASTAPI-API</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Backend Servidor API REST</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Gestión de endpoints de inferencia de telemetría de gases, búfer circular en vivo y persistencia de lifespan de modelos.</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>fastapi_server/api.py
 fastapi_server/requirements.txt</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>070c6f3</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>fastapi_server/test_api.py</t>
         </is>
       </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>Endpoints REST HTTP 200/400 validados con Pytest</t>
         </is>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
         <is>
           <t>APROBADO</t>
         </is>
@@ -794,7 +807,7 @@
           <t>main</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>ae596a0</t>
         </is>
@@ -809,55 +822,55 @@
           <t>Diseño responsivo móvil y anti-flicker HTML5 validado</t>
         </is>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="I10" s="12" t="inlineStr">
         <is>
           <t>APROBADO</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>BOLT-004-LCD-CLIENT</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>Hardware LCD e Iniciar Servicio</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>Cliente IoT autónomo para pantalla física LCD 16x2 I2C con refresco de caché anti-parpadeo y daemon de arranque automático.</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>fastapi_server/lcd_client.py
 fastapi_server/start_enose.sh</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="F11" s="18" t="inlineStr">
         <is>
           <t>039f8bd</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>Emulación local en consola e integración física por hardware</t>
         </is>
       </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="H11" s="15" t="inlineStr">
         <is>
           <t>Pantalla LCD 16x2 I2C I/O estable en bus I2C (dirección 0x27)</t>
         </is>
       </c>
-      <c r="I11" s="11" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>APROBADO</t>
         </is>
@@ -890,7 +903,7 @@
           <t>main</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>5466a92</t>
         </is>
@@ -905,29 +918,29 @@
           <t>Envío exitoso de tramas a velocidad de muestreo estable</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr">
         <is>
           <t>APROBADO</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>BOLT-006-TEST-SUITE</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Aseguramiento de Calidad QA</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>Suite unificada de pruebas unitarias, análisis estático para SonarQube e integración de calidad con reporte de cobertura XML.</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>run_all_tests.py
 fastapi_server/sonar-project.properties
@@ -935,28 +948,28 @@
 doc_investigacion_y_pruebas.md</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
+      <c r="F13" s="18" t="inlineStr">
         <is>
           <t>ed283a6</t>
         </is>
       </c>
-      <c r="G13" s="15" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>run_all_tests.py ( pytest + pytest-cov )</t>
         </is>
       </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="15" t="inlineStr">
         <is>
           <t>92.0% Cobertura de código
 0 Bugs críticos de código</t>
         </is>
       </c>
-      <c r="I13" s="11" t="inlineStr">
+      <c r="I13" s="12" t="inlineStr">
         <is>
           <t>APROBADO</t>
         </is>
@@ -970,6 +983,14 @@
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="F5:I5"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
QA: Reemplazo de hashes cortos por URLs de commits completas en la matriz de control de versiones
</commit_message>
<xml_diff>
--- a/Matriz_Registro_Control_de_Versiones.xlsx
+++ b/Matriz_Registro_Control_de_Versiones.xlsx
@@ -72,7 +72,6 @@
     </font>
     <font>
       <name val="Consolas"/>
-      <b val="1"/>
       <color rgb="000d6efd"/>
       <sz val="9"/>
       <u val="single"/>
@@ -565,7 +564,7 @@
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
     <col width="35" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
@@ -713,7 +712,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>0629d31</t>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/0629d31</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -762,7 +761,7 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>070c6f3</t>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/070c6f3</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
@@ -809,7 +808,7 @@
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>ae596a0</t>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/ae596a0</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -857,7 +856,7 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>039f8bd</t>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/039f8bd</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
@@ -905,7 +904,7 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>5466a92</t>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/5466a92</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -955,7 +954,7 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>ed283a6</t>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/ed283a6</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">

</xml_diff>